<commit_message>
D83-D84: drop art & design from the Test B question; week of 28 Sep for Test E; screens page to D81
- Art & design removed from the Test A question, aspiration.yaml, tests and
  the results-sheet note (recalculated: 4,100 formulas, 0 errors, no cell
  changed); parked on decisions/after-9-nov.md.
- First 2 Test E interviews in the week of 28 Sep if contacts reply; the
  Areas 5-7 review parked after 9 Nov; ~5 h of that week kept as buffer.
- LOG totals: 112 h scheduled (8 h parked), about 0.9 weeks past the window.
- v0-ios-plan points to LOG.md for the weekly schedule.
- Published screens page updated to D81 (4 custom screens, rest native).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UzWNUrDcAUTEJSyAB9gGKc
</commit_message>
<xml_diff>
--- a/validation/results-sheet.xlsx
+++ b/validation/results-sheet.xlsx
@@ -43,7 +43,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Test A question 5.7 (D77), optional. Enter the fields they picked, comma-separated: finance &amp; tech, food, history &amp; culture, nature, art &amp; design. Enter 'none' for none of these; leave blank if skipped. Read by brain.testb.</t>
+          <t xml:space="preserve">Test A question 5.7 (D77), optional. Enter the fields they picked, comma-separated: finance &amp; tech, food, history &amp; culture, nature. Enter 'none' for none of these; leave blank if skipped. Art &amp; design was dropped for Test B (D83). Read by brain.testb.</t>
         </r>
       </text>
     </comment>
@@ -5356,7 +5356,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="1" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="32" min="21" style="1" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="1" width="24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>